<commit_message>
PPT - 17/06/2026 - vers2
</commit_message>
<xml_diff>
--- a/dashboard_data_template.xlsx
+++ b/dashboard_data_template.xlsx
@@ -473,13 +473,13 @@
         <v>Creación de Solución</v>
       </c>
       <c r="F2" t="str">
-        <v>"- Opciones de interfaces compartidas por S3:</v>
+        <v>- Opciones de interfaces compartidas por S3: CGC Position, Valorized Position, Net Asset, Payable Receivable - La POC ha sido presentada.</v>
       </c>
       <c r="G2" t="str">
         <v>09/04/2026</v>
       </c>
       <c r="H2" t="str">
-        <v>-----------------------</v>
+        <v>-----------------------_x000d_</v>
       </c>
     </row>
     <row r="3">
@@ -713,7 +713,7 @@
         <v>27/05/2026</v>
       </c>
       <c r="H11" t="str">
-        <v>- NFQ ajustara segun el orden de prioridad de tareas_x000d_</v>
+        <v>- NFQ ajustara segun el orden de prioridad de tarefas_x000d_</v>
       </c>
     </row>
     <row r="12">
@@ -739,7 +739,7 @@
         <v>17/06/2026</v>
       </c>
       <c r="H12" t="str">
-        <v>- NFQ ajustara segun el orden de prioridad de tareas</v>
+        <v>- NFQ ajustara segun el orden de prioridad de tarefas</v>
       </c>
     </row>
   </sheetData>
@@ -809,25 +809,25 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Nuevos reportes</v>
+        <v>Completado</v>
       </c>
       <c r="B2" t="str">
-        <v>Completado</v>
+        <v>PRD</v>
       </c>
       <c r="C2" t="str">
-        <v>PRD</v>
+        <v>NFQ / S3</v>
       </c>
       <c r="D2" t="str">
-        <v>NFQ / S3</v>
+        <v>Creación de reporte: Relatório de Estoque de Cotas de Fundos</v>
       </c>
       <c r="E2" t="str">
-        <v>Creación de reporte: Relatório de Estoque de Cotas de Fundos</v>
+        <v>- Informe Disponibilizado en PRD</v>
       </c>
       <c r="F2" t="str">
-        <v>- Informe Disponibilizado en PRD</v>
+        <v>27/05/2026</v>
       </c>
       <c r="G2" t="str">
-        <v>27/05/2026</v>
+        <v>- S3 validará desarrollo_x000d_</v>
       </c>
       <c r="H2" t="str">
         <v>- S3 validará desarrollo_x000d_</v>
@@ -835,25 +835,25 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Nuevos reportes</v>
+        <v>Completado</v>
       </c>
       <c r="B3" t="str">
-        <v>Completado</v>
+        <v>PRD</v>
       </c>
       <c r="C3" t="str">
-        <v>PRD</v>
+        <v>NFQ / S3</v>
       </c>
       <c r="D3" t="str">
-        <v>NFQ / S3</v>
+        <v>Creación de reporte: Relatório de Estoque de Futuros</v>
       </c>
       <c r="E3" t="str">
-        <v>Creación de reporte: Relatório de Estoque de Futuros</v>
+        <v>- Informe Disponibilizado en PRD</v>
       </c>
       <c r="F3" t="str">
-        <v>- Informe Disponibilizado en PRD</v>
+        <v>27/05/2026</v>
       </c>
       <c r="G3" t="str">
-        <v>27/05/2026</v>
+        <v>- S3 validará desarrollo_x000d_</v>
       </c>
       <c r="H3" t="str">
         <v>- S3 validará desarrollo_x000d_</v>
@@ -861,25 +861,25 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Nuevos reportes</v>
+        <v>Completado</v>
       </c>
       <c r="B4" t="str">
-        <v>Completado</v>
+        <v>PRD</v>
       </c>
       <c r="C4" t="str">
-        <v>PRD</v>
+        <v>NFQ / S3</v>
       </c>
       <c r="D4" t="str">
-        <v>NFQ / S3</v>
+        <v>Creación de reporte: Relatório de Estoque de RV</v>
       </c>
       <c r="E4" t="str">
-        <v>Creación de reporte: Relatório de Estoque de RV</v>
+        <v>- Informe Disponibilizado en PRD</v>
       </c>
       <c r="F4" t="str">
-        <v>- Informe Disponibilizado en PRD</v>
+        <v>03/06/2026</v>
       </c>
       <c r="G4" t="str">
-        <v>03/06/2026</v>
+        <v>- S3 validará desarrollo_x000d_</v>
       </c>
       <c r="H4" t="str">
         <v>- S3 validará desarrollo_x000d_</v>
@@ -887,25 +887,25 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Nuevos reportes</v>
+        <v>Completado</v>
       </c>
       <c r="B5" t="str">
-        <v>Completado</v>
+        <v>PRD</v>
       </c>
       <c r="C5" t="str">
-        <v>PRD</v>
+        <v>NFQ / S3</v>
       </c>
       <c r="D5" t="str">
-        <v>NFQ / S3</v>
+        <v>Creación de reporte: Relatório de Estoque de RF</v>
       </c>
       <c r="E5" t="str">
-        <v>Creación de reporte: Relatório de Estoque de RF</v>
+        <v>- Informe Disponibilizado en PRD</v>
       </c>
       <c r="F5" t="str">
-        <v>- Informe Disponibilizado en PRD</v>
+        <v>27/05/2026</v>
       </c>
       <c r="G5" t="str">
-        <v>27/05/2026</v>
+        <v>- S3 validará desarrollo_x000d_</v>
       </c>
       <c r="H5" t="str">
         <v>- S3 validará desarrollo_x000d_</v>
@@ -913,25 +913,25 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Demonstrativo de caixa</v>
+        <v>Completado</v>
       </c>
       <c r="B6" t="str">
-        <v>Completado</v>
+        <v>PRD</v>
       </c>
       <c r="C6" t="str">
-        <v>PRD</v>
+        <v>S3 / NFQ / VERMEG</v>
       </c>
       <c r="D6" t="str">
-        <v>S3 / NFQ / VERMEG</v>
+        <v>Saldos</v>
       </c>
       <c r="E6" t="str">
-        <v>Saldos</v>
+        <v>- Vermeg ha modificado la configuración de SupervisionDashboard en PRD para que se ejecute a las 06:00 (Horário de Brasilia)</v>
       </c>
       <c r="F6" t="str">
-        <v>- Vermeg ha modificado la configuración de SupervisionDashboard en PRD para que se ejecute a las 06:00 (Horário de Brasilia)</v>
+        <v>18/05/2026</v>
       </c>
       <c r="G6" t="str">
-        <v>18/05/2026</v>
+        <v>NA_x000d_</v>
       </c>
       <c r="H6" t="str">
         <v>NA_x000d_</v>
@@ -939,25 +939,25 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Operações com Título de Renda Fixa</v>
+        <v>En proceso</v>
       </c>
       <c r="B7" t="str">
-        <v>En proceso</v>
+        <v>PRD</v>
       </c>
       <c r="C7" t="str">
-        <v>PRD</v>
+        <v>S3 / NFQ / VERMEG</v>
       </c>
       <c r="D7" t="str">
-        <v>S3 / NFQ / VERMEG</v>
+        <v>Reglas</v>
       </c>
       <c r="E7" t="str">
-        <v>Reglas</v>
+        <v>- Se ha ajustado la regla de visualización de los saldos de los fondos MEGARA.</v>
       </c>
       <c r="F7" t="str">
-        <v>- Se ha ajustado la regla de visualización de los saldos de los fondos MEGARA.</v>
+        <v>10/06/2026</v>
       </c>
       <c r="G7" t="str">
-        <v>10/06/2026</v>
+        <v>- Se realizará desarrollo segun orden de priorización</v>
       </c>
       <c r="H7" t="str">
         <v>- Se realizará desarrollo segun orden de priorización</v>
@@ -1071,7 +1071,7 @@
         <v>Llamada de MEGARA desde Rundeck</v>
       </c>
       <c r="F3" t="str">
-        <v>"- NFQ ha implementado solución y se encuentra operativa en PRD</v>
+        <v>- NFQ ha implementado solución y se encuentra operativa en PRD - Fallas ocasionaes de lado de Megara (Durante la implementación de las interfaces, Megacustody se bloqueó) - La activación manual de Scheduled Megara mientras la API estaba activada ha provocado problemas</v>
       </c>
       <c r="G3" t="str">
         <v>24/3/2026</v>
@@ -1089,7 +1089,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H16"/>
   <cols>
     <col min="1" max="1" width="50.00390625" customWidth="1"/>
     <col min="2" max="2" width="17.83203125" customWidth="1"/>
@@ -1147,129 +1147,129 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Detalhado de Estoque de RF_x000d_</v>
+        <v>Detalhado de Estoque de RF</v>
       </c>
       <c r="B2" t="str">
-        <v>En proceso_x000d_</v>
+        <v>En proceso</v>
       </c>
       <c r="C2" t="str">
         <v>PRD</v>
       </c>
       <c r="D2" t="str">
-        <v>S3 / NFQ_x000d_</v>
+        <v>S3 / NFQ</v>
       </c>
       <c r="E2" t="str">
-        <v>Ajuste_x000d_</v>
+        <v>Ajuste</v>
       </c>
       <c r="F2" t="str">
-        <v>"- Ajuste de reglas para campos de Lucro / Prejuizo - S3 en validación de ajustes hechos por NFQ"</v>
+        <v>- Ajuste de reglas para campos de Lucro / Prejuizo - S3 en validación de ajustes hechos por NFQ</v>
       </c>
       <c r="G2" t="str">
-        <v>03/04/2026_x000d_</v>
+        <v>03/04/2026</v>
       </c>
       <c r="H2" t="str">
-        <v>Aguardando validacion de S3.</v>
+        <v>Aguardando validacion de S3._x000d_</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Extrato Simplificado_x000d_</v>
+        <v>Extrato Simplificado</v>
       </c>
       <c r="B3" t="str">
-        <v>En proceso_x000d_</v>
+        <v>En proceso</v>
       </c>
       <c r="C3" t="str">
         <v>PRD</v>
       </c>
       <c r="D3" t="str">
-        <v>S3 / NFQ_x000d_</v>
+        <v>S3 / NFQ</v>
       </c>
       <c r="E3" t="str">
-        <v>Desarrollo_x000d_</v>
+        <v>Desarrollo</v>
       </c>
       <c r="F3" t="str">
-        <v>"- S3 ha validado PDF y XLSX - - Liberado en UAT, a la espera de promocion en PRD - - A la espera que S3 comparta plantilla de CSV"</v>
+        <v>- S3 ha validado PDF y XLSX - Liberado en UAT, a la espera de promocion en PRD - A la espera que S3 comparta plantilla de CSV</v>
       </c>
       <c r="G3" t="str">
-        <v>29/04/2026_x000d_</v>
+        <v>29/04/2026</v>
       </c>
       <c r="H3" t="str">
-        <v>"-S3 compartirá template en csv. - -NFQ ya ha vuelto a solicitar a S3 que envíe los archivos"</v>
+        <v>-S3 compartirá template en csv. -NFQ ya ha vuelto a solicitar a S3 que envíe los arquivos_x000d_</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Informes Asíncronos_x000d_</v>
+        <v>Informes Asíncronos</v>
       </c>
       <c r="B4" t="str">
-        <v>En proceso_x000d_</v>
+        <v>En proceso</v>
       </c>
       <c r="C4" t="str">
         <v>PRD</v>
       </c>
       <c r="D4" t="str">
-        <v>NTT / NFQ / VERMEG_x000d_</v>
+        <v>NTT / NFQ / VERMEG</v>
       </c>
       <c r="E4" t="str">
-        <v>S3 solicita la creación de informes asíncronos_x000d_</v>
+        <v>S3 solicita la creación de informes asíncronos</v>
       </c>
       <c r="F4" t="str">
-        <v>"- NFQ ha compartido calendario de entrega para los informes solicitados. - - Testes OK de (Fluxo de Caixa, Operacoes Títulos RF) - - Espernando repuesta de Operacoes com Titulos de Renda Variavel - - NFQ en desarrollo de 1 informe (Extrato Simplificado)"</v>
+        <v>- NFQ ha compartido calendario de entrega para los informes solicitados. - Testes OK de (Fluxo de Caixa, Operacoes Títulos RF) - Espernando repuesta de Operacoes com Titulos de Renda Variavel - NFQ en desarrollo de 1 informe (Extrato Simplificado)</v>
       </c>
       <c r="G4" t="str">
-        <v>22/04/2026_x000d_</v>
+        <v>22/04/2026</v>
       </c>
       <c r="H4" t="str">
-        <v>"Espernado respuesta de Operaciones de Titulos ed Renda Variavel (cliente y fecha) - S3 entregará informes de Extrato Simplifcado"</v>
+        <v>Espernado respuesta de Operaciones de Titulos ed Renda Variavel (cliente y fecha) S3 entregará informes de Extrato Simplifcado_x000d_</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Nuevas Interfaces_x000d_</v>
+        <v>Nuevas Interfaces</v>
       </c>
       <c r="B5" t="str">
-        <v>En proceso_x000d_</v>
+        <v>En proceso</v>
       </c>
       <c r="C5" t="str">
         <v>PRD</v>
       </c>
       <c r="D5" t="str">
-        <v>NFQ / S3_x000d_</v>
+        <v>NFQ / S3</v>
       </c>
       <c r="E5" t="str">
-        <v>"Creación de 2 nuevas interfaces (Recalculation_Request, RecalculationRequest Reason)</v>
+        <v>Creación de 2 nuevas interfaces (Recalculation_Request, Recalculation_Request_Reason)</v>
       </c>
       <c r="F5" t="str">
         <v>- Desarrollo realizado en UAT.</v>
       </c>
       <c r="G5" t="str">
-        <v>29/04/2026_x000d_</v>
+        <v>29/04/2026</v>
       </c>
       <c r="H5" t="str">
-        <v>- Validación de lado S3 para pomocionar a UAT_x000d_</v>
+        <v>- Validación de lado S3 para promocionar a UAT_x000d_</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Mapeo_x000d_</v>
+        <v>Mapeo</v>
       </c>
       <c r="B6" t="str">
-        <v>⚠️_x000d_</v>
+        <v>⚠️UAT</v>
       </c>
       <c r="C6" t="str">
-        <v>UAT</v>
+        <v>S3</v>
       </c>
       <c r="D6" t="str">
-        <v>S3_x000d_</v>
+        <v>Validación ajuste en UAT function_meg_sac_stat_cli_addr_t</v>
       </c>
       <c r="E6" t="str">
-        <v>Validación ajuste en UAT function_meg_sac_stat_cli_addr_t_x000d_</v>
+        <v>- En espera de validación por parte de S3 para promoción a PRD.</v>
       </c>
       <c r="F6" t="str">
         <v>- En espera de validación por parte de S3 para promoción a PRD.</v>
       </c>
       <c r="G6" t="str">
-        <v>07/07/2025_x000d_</v>
+        <v>07/07/2025</v>
       </c>
       <c r="H6" t="str">
         <v>Validación de lado S3_x000d_</v>
@@ -1277,25 +1277,25 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>DDBB_x000d_</v>
+        <v>DDBB</v>
       </c>
       <c r="B7" t="str">
-        <v>⚠️_x000d_</v>
+        <v>⚠️UAT</v>
       </c>
       <c r="C7" t="str">
-        <v>UAT</v>
+        <v>S3</v>
       </c>
       <c r="D7" t="str">
-        <v>S3_x000d_</v>
+        <v>CA_details_intr</v>
       </c>
       <c r="E7" t="str">
-        <v>CA_details_intr_x000d_</v>
+        <v>- Ajuste de formatos de datos</v>
       </c>
       <c r="F7" t="str">
         <v>- Ajuste de formatos de datos_x000d_</v>
       </c>
       <c r="G7" t="str">
-        <v>05/09/2025_x000d_</v>
+        <v>05/09/2025</v>
       </c>
       <c r="H7" t="str">
         <v>Validación de lado S3_x000d_</v>
@@ -1303,25 +1303,25 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Creación mapeos_x000d_</v>
+        <v>Creación mapeos</v>
       </c>
       <c r="B8" t="str">
-        <v>⚠️_x000d_</v>
+        <v>⚠️UAT</v>
       </c>
       <c r="C8" t="str">
-        <v>UAT</v>
+        <v>NFQ / S3</v>
       </c>
       <c r="D8" t="str">
-        <v>NFQ / S3_x000d_</v>
+        <v>Nuevos Mapeos</v>
       </c>
       <c r="E8" t="str">
-        <v>Nuevos Mapeos_x000d_</v>
+        <v>-Se encuentra en development 3 novos mapeos que utilizaran la extracción InvestCompanyInstitute</v>
       </c>
       <c r="F8" t="str">
         <v>-Se encuentra en desarrollo 3 nuevos mapeos que utilizaran la extracción InvestCompanyInstitute_x000d_</v>
       </c>
       <c r="G8" t="str">
-        <v>28/10/2025_x000d_</v>
+        <v>28/10/2025</v>
       </c>
       <c r="H8" t="str">
         <v>Validación de lado S3_x000d_</v>
@@ -1329,25 +1329,25 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Ajuste InvestCompanyInstitute_x000d_</v>
+        <v>Ajuste InvestCompanyInstitute</v>
       </c>
       <c r="B9" t="str">
-        <v>⚠️_x000d_</v>
+        <v>⚠️UAT</v>
       </c>
       <c r="C9" t="str">
-        <v>UAT</v>
+        <v>NFQ / S3 / Vermeg / NTT</v>
       </c>
       <c r="D9" t="str">
-        <v>NFQ / S3 / Vermeg / NTT_x000d_</v>
+        <v>Subtabla</v>
       </c>
       <c r="E9" t="str">
-        <v>Subtabla_x000d_</v>
+        <v>-Se incluyó una nueva subtabla dentro del XSD, se construyó y promocionó a UAT, a espera de validación de S3</v>
       </c>
       <c r="F9" t="str">
         <v>-Se incluyó una nueva subtabla dentro del XSD, se construyó y promocionó a UAT, a espera de validación de S3</v>
       </c>
       <c r="G9" t="str">
-        <v>28/10/2025_x000d_</v>
+        <v>28/10/2025</v>
       </c>
       <c r="H9" t="str">
         <v>Validación de lado S3_x000d_</v>
@@ -1355,25 +1355,25 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Mapeo_x000d_</v>
+        <v>Mapeo</v>
       </c>
       <c r="B10" t="str">
-        <v>❗_x000d_</v>
+        <v>❗PRD</v>
       </c>
       <c r="C10" t="str">
-        <v>PRD</v>
+        <v>NFQ / S3</v>
       </c>
       <c r="D10" t="str">
-        <v>NFQ / S3_x000d_</v>
+        <v>Errores ejecución de Mapeo</v>
       </c>
       <c r="E10" t="str">
-        <v>Errores ejecución de Mapeo_x000d_</v>
+        <v>- mt_caixa_tipos (longitud de campo) value too long for type character varying(50) - Ajuste en UAT conforme acordado, en espera de confirmación por parte de S3 para promoción a producción.</v>
       </c>
       <c r="F10" t="str">
-        <v>"- mt_caixa_tipos (longitud de campo) - value too long for type character varying(50) - - Ajuste en UAT conforme acordado, en espera de confirmación por parte de S3 para promoción a producción."</v>
+        <v>- mt_caixa_tipos (longitud de campo) value too long for type character varying(50) - Ajuste en UAT conforme acordado, en espera de confirmación por parte de S3 para promoción a producción.</v>
       </c>
       <c r="G10" t="str">
-        <v>31/10/2025_x000d_</v>
+        <v>31/10/2025</v>
       </c>
       <c r="H10" t="str">
         <v>Validación de lado S3_x000d_</v>
@@ -1381,25 +1381,25 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Ajuste Proceso de Carga_x000d_</v>
+        <v>Ajuste Proceso de Carga</v>
       </c>
       <c r="B11" t="str">
-        <v>⚠️_x000d_</v>
+        <v>⚠️UAT</v>
       </c>
       <c r="C11" t="str">
-        <v>UAT</v>
+        <v>NFQ / S3</v>
       </c>
       <c r="D11" t="str">
-        <v>NFQ / S3_x000d_</v>
+        <v>Ajuste de Interfaz Equity</v>
       </c>
       <c r="E11" t="str">
-        <v>Ajuste de Interfaz Equity_x000d_</v>
+        <v>- Fue incluido un nuevo campo, a espera de validación y promoción a PRD</v>
       </c>
       <c r="F11" t="str">
         <v>- Fue incluido un nuevo campo, a espera de validación y promoción a PRD_x000d_</v>
       </c>
       <c r="G11" t="str">
-        <v>21/01/2026_x000d_</v>
+        <v>21/01/2026</v>
       </c>
       <c r="H11" t="str">
         <v>Validación de lado S3_x000d_</v>
@@ -1407,25 +1407,25 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Ajuste Proceso de Carga_x000d_</v>
+        <v>Ajuste Proceso de Carga</v>
       </c>
       <c r="B12" t="str">
-        <v>⚠️_x000d_</v>
+        <v>⚠️UAT</v>
       </c>
       <c r="C12" t="str">
-        <v>UAT</v>
+        <v>NFQ / S3</v>
       </c>
       <c r="D12" t="str">
-        <v>NFQ / S3_x000d_</v>
+        <v>Ajuste de Carga ScriptByClient</v>
       </c>
       <c r="E12" t="str">
-        <v>Ajuste de Carga ScriptByClient_x000d_</v>
+        <v>- Fue realizado un ajuste en la carga de las tablas Megara que alimentan el mapeo SAC_BA_SCRIPT</v>
       </c>
       <c r="F12" t="str">
         <v>- Fue realizado un ajuste en la carga de las tablas Megara que alimentan el mapeo SAC_BA_SCRIPT_x000d_</v>
       </c>
       <c r="G12" t="str">
-        <v>28/01/2026_x000d_</v>
+        <v>28/01/2026</v>
       </c>
       <c r="H12" t="str">
         <v>Validación de lado S3_x000d_</v>
@@ -1433,80 +1433,80 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Información UAT_x000d_</v>
+        <v>Información UAT</v>
       </c>
       <c r="B13" t="str">
-        <v>⚫_x000d_</v>
+        <v>⚫UAT</v>
       </c>
       <c r="C13" t="str">
-        <v>UAT</v>
+        <v>NFQ / S3</v>
       </c>
       <c r="D13" t="str">
-        <v>NFQ / S3_x000d_</v>
+        <v>Monitoreamento de cargas</v>
       </c>
       <c r="E13" t="str">
-        <v>Monitoreamento de cargas_x000d_</v>
+        <v>- Se requerirá de validaciones de informação por causa de los mapeos en UAT</v>
       </c>
       <c r="F13" t="str">
         <v>- Se requerirá de validaciones de información por causa de los mapeos en UAT_x000d_</v>
       </c>
       <c r="G13" t="str">
-        <v>31/10/2025_x000d_</v>
+        <v>31/10/2025</v>
       </c>
       <c r="H13" t="str">
-        <v>- S3 junto con NFQ revisará ambiente, a la espera de activación al equipo de proyecto_x000d_</v>
+        <v>- S3 junto con NFQ revisará ambiente, a la espera de activación al equipo de projeto_x000d_</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Datahub Api_x000d_</v>
+        <v>Datahub Api</v>
       </c>
       <c r="B14" t="str">
-        <v>▶️_x000d_</v>
+        <v>▶️UAT</v>
       </c>
       <c r="C14" t="str">
-        <v>UAT</v>
+        <v>NFQ / S3</v>
       </c>
       <c r="D14" t="str">
-        <v>NFQ / S3_x000d_</v>
+        <v>dh-motivobloqueio</v>
       </c>
       <c r="E14" t="str">
-        <v>dh-motivobloqueio_x000d_</v>
+        <v>- Api Motivo de Bloqueos han sido realizados los ajustes y está pendiente validación por parte de S3</v>
       </c>
       <c r="F14" t="str">
         <v>- Api Motivo de Bloqueos han sido realizados los ajustes y está pendiente validación por parte de S3</v>
       </c>
       <c r="G14" t="str">
-        <v>21/01/2026_x000d_</v>
+        <v>21/01/2026</v>
       </c>
       <c r="H14" t="str">
-        <v>- S3 notificará resultados de validaciones</v>
+        <v>- S3 notificará resultados de validaciones_x000d_</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Generacion informes_x000d_</v>
+        <v>Generacion informes</v>
       </c>
       <c r="B15" t="str">
-        <v>▶️_x000d_</v>
+        <v>▶️PRD</v>
       </c>
       <c r="C15" t="str">
-        <v>PRD</v>
+        <v>S3 / NFQ</v>
       </c>
       <c r="D15" t="str">
-        <v>S3 / NFQ_x000d_</v>
+        <v>Revisión de informes vacos</v>
       </c>
       <c r="E15" t="str">
-        <v>Revisión de informes vacos_x000d_</v>
+        <v>- Movimentaçao Swap, Dividendos juros apropiados, Posiçao Swap siendo generados en blanco. - Primeros dos arreglados, esperando detalles del tercero.</v>
       </c>
       <c r="F15" t="str">
-        <v>"- Movimentaçao Swap, Dividendos juros apropiados,Posiçao Swap.siendo generados en blanco. - - Primeros dos arreglados, esperando detalles del tercero.</v>
+        <v>- Movimentaçao Swap, Dividendos juros apropiados, Posiçao Swap siendo generados en blanco. - Primeros dos arreglados, esperando detalles del tercero.</v>
       </c>
       <c r="G15" t="str">
-        <v>29/01/2026_x000d_</v>
+        <v>29/01/2026</v>
       </c>
       <c r="H15" t="str">
-        <v>"- S3 validará arreglos en los informes. - - S3 compartirá detalles de PS para poder dar soporte."</v>
+        <v>- S3 validará arreglos en los informes. - S3 compartirá detalles de PS para poder dar suporte._x000d_</v>
       </c>
     </row>
     <row r="16">
@@ -1514,19 +1514,19 @@
         <v>Nota de Liquidaçao de Renda Fixa</v>
       </c>
       <c r="B16" t="str">
-        <v>▶️</v>
+        <v>▶️PRD</v>
       </c>
       <c r="C16" t="str">
-        <v>PRD</v>
+        <v>S3 / NFQ</v>
       </c>
       <c r="D16" t="str">
-        <v>S3 / NFQ</v>
+        <v>Generación de informe</v>
       </c>
       <c r="E16" t="str">
-        <v>Generación de informe</v>
+        <v>- S3 en análisis de cambio de plantilla para casos sin información. - S3 reporta error en generación de informe. - NFQ hizo ajustes.</v>
       </c>
       <c r="F16" t="str">
-        <v>"- S3 en análisis de cambio de plantilla para casos sin información. - - S3 reporta error en generación de informe. - - NFQ hizo ajustes."</v>
+        <v>- S3 en análisis de cambio de plantilla para casos sin información. - S3 reporta error en generación de informe. - NFQ hizo ajustes.</v>
       </c>
       <c r="G16" t="str">
         <v>09/02/2026</v>
@@ -1535,14 +1535,9 @@
         <v>- S3 analizará cambio de plantilla</v>
       </c>
     </row>
-    <row r="17">
-      <c r="E17" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
PPT 17/06/2026 - Arreglado
</commit_message>
<xml_diff>
--- a/dashboard_data_template.xlsx
+++ b/dashboard_data_template.xlsx
@@ -402,14 +402,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H12"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" customWidth="1"/>
-    <col min="5" max="5" width="16.6640625" customWidth="1"/>
-    <col min="6" max="6" width="16.6640625" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" customWidth="1"/>
-    <col min="8" max="8" width="16.6640625" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="20.33203125" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" customWidth="1"/>
+    <col min="7" max="7" width="20.33203125" customWidth="1"/>
+    <col min="8" max="8" width="20.33203125" customWidth="1"/>
     <col min="9" max="9" width="16.6640625" customWidth="1"/>
     <col min="10" max="10" width="16.6640625" customWidth="1"/>
     <col min="11" max="11" width="16.6640625" customWidth="1"/>
@@ -479,7 +479,7 @@
         <v>09/04/2026</v>
       </c>
       <c r="H2" t="str">
-        <v>-----------------------_x000d_</v>
+        <v>-----------------------</v>
       </c>
     </row>
     <row r="3">
@@ -635,7 +635,7 @@
         <v>10/06/2026</v>
       </c>
       <c r="H8" t="str">
-        <v>- S3 validará desarrollo_x000d_</v>
+        <v>- S3 validará desarrollo</v>
       </c>
     </row>
     <row r="9">
@@ -661,7 +661,7 @@
         <v>15/06/2026</v>
       </c>
       <c r="H9" t="str">
-        <v>- S3 validará desarrollo_x000d_</v>
+        <v>- S3 validará desarrollo</v>
       </c>
     </row>
     <row r="10">
@@ -687,7 +687,7 @@
         <v>17/06/2026</v>
       </c>
       <c r="H10" t="str">
-        <v>- S3 validará desarrollo_x000d_</v>
+        <v>- S3 validará desarrollo</v>
       </c>
     </row>
     <row r="11">
@@ -713,7 +713,7 @@
         <v>27/05/2026</v>
       </c>
       <c r="H11" t="str">
-        <v>- NFQ ajustara segun el orden de prioridad de tarefas_x000d_</v>
+        <v>- NFQ ajustara segun el orden de prioridad de tarefas</v>
       </c>
     </row>
     <row r="12">
@@ -753,14 +753,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H7"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" customWidth="1"/>
-    <col min="5" max="5" width="16.6640625" customWidth="1"/>
-    <col min="6" max="6" width="16.6640625" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" customWidth="1"/>
-    <col min="8" max="8" width="16.6640625" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="20.33203125" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" customWidth="1"/>
+    <col min="7" max="7" width="20.33203125" customWidth="1"/>
+    <col min="8" max="8" width="20.33203125" customWidth="1"/>
     <col min="9" max="9" width="16.6640625" customWidth="1"/>
     <col min="10" max="10" width="16.6640625" customWidth="1"/>
     <col min="11" max="11" width="16.6640625" customWidth="1"/>
@@ -809,155 +809,155 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>Nuevos reportes</v>
+      </c>
+      <c r="B2" t="str">
         <v>Completado</v>
       </c>
-      <c r="B2" t="str">
-        <v>PRD</v>
-      </c>
       <c r="C2" t="str">
-        <v>NFQ / S3</v>
+        <v>PRD</v>
       </c>
       <c r="D2" t="str">
+        <v>NFQ / S3</v>
+      </c>
+      <c r="E2" t="str">
         <v>Creación de reporte: Relatório de Estoque de Cotas de Fundos</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>- Informe Disponibilizado en PRD</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>27/05/2026</v>
       </c>
-      <c r="G2" t="str">
-        <v>- S3 validará desarrollo_x000d_</v>
-      </c>
       <c r="H2" t="str">
-        <v>- S3 validará desarrollo_x000d_</v>
+        <v>- S3 validará desarrollo</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>Nuevos reportes</v>
+      </c>
+      <c r="B3" t="str">
         <v>Completado</v>
       </c>
-      <c r="B3" t="str">
-        <v>PRD</v>
-      </c>
       <c r="C3" t="str">
-        <v>NFQ / S3</v>
+        <v>PRD</v>
       </c>
       <c r="D3" t="str">
+        <v>NFQ / S3</v>
+      </c>
+      <c r="E3" t="str">
         <v>Creación de reporte: Relatório de Estoque de Futuros</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>- Informe Disponibilizado en PRD</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>27/05/2026</v>
       </c>
-      <c r="G3" t="str">
-        <v>- S3 validará desarrollo_x000d_</v>
-      </c>
       <c r="H3" t="str">
-        <v>- S3 validará desarrollo_x000d_</v>
+        <v>- S3 validará desarrollo</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>Nuevos reportes</v>
+      </c>
+      <c r="B4" t="str">
         <v>Completado</v>
       </c>
-      <c r="B4" t="str">
-        <v>PRD</v>
-      </c>
       <c r="C4" t="str">
-        <v>NFQ / S3</v>
+        <v>PRD</v>
       </c>
       <c r="D4" t="str">
+        <v>NFQ / S3</v>
+      </c>
+      <c r="E4" t="str">
         <v>Creación de reporte: Relatório de Estoque de RV</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>- Informe Disponibilizado en PRD</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>03/06/2026</v>
       </c>
-      <c r="G4" t="str">
-        <v>- S3 validará desarrollo_x000d_</v>
-      </c>
       <c r="H4" t="str">
-        <v>- S3 validará desarrollo_x000d_</v>
+        <v>- S3 validará desarrollo</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>Nuevos reportes</v>
+      </c>
+      <c r="B5" t="str">
         <v>Completado</v>
       </c>
-      <c r="B5" t="str">
-        <v>PRD</v>
-      </c>
       <c r="C5" t="str">
-        <v>NFQ / S3</v>
+        <v>PRD</v>
       </c>
       <c r="D5" t="str">
+        <v>NFQ / S3</v>
+      </c>
+      <c r="E5" t="str">
         <v>Creación de reporte: Relatório de Estoque de RF</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>- Informe Disponibilizado en PRD</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>27/05/2026</v>
       </c>
-      <c r="G5" t="str">
-        <v>- S3 validará desarrollo_x000d_</v>
-      </c>
       <c r="H5" t="str">
-        <v>- S3 validará desarrollo_x000d_</v>
+        <v>- S3 validará desarrollo</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>Demonstrativo de caixa</v>
+      </c>
+      <c r="B6" t="str">
         <v>Completado</v>
       </c>
-      <c r="B6" t="str">
-        <v>PRD</v>
-      </c>
       <c r="C6" t="str">
+        <v>PRD</v>
+      </c>
+      <c r="D6" t="str">
         <v>S3 / NFQ / VERMEG</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>Saldos</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>- Vermeg ha modificado la configuración de SupervisionDashboard en PRD para que se ejecute a las 06:00 (Horário de Brasilia)</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>18/05/2026</v>
       </c>
-      <c r="G6" t="str">
-        <v>NA_x000d_</v>
-      </c>
       <c r="H6" t="str">
-        <v>NA_x000d_</v>
+        <v>NA</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>Operações com Título de Renda Fixa</v>
+      </c>
+      <c r="B7" t="str">
         <v>En proceso</v>
       </c>
-      <c r="B7" t="str">
-        <v>PRD</v>
-      </c>
       <c r="C7" t="str">
+        <v>PRD</v>
+      </c>
+      <c r="D7" t="str">
         <v>S3 / NFQ / VERMEG</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>Reglas</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <v>- Se ha ajustado la regla de visualización de los saldos de los fondos MEGARA.</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>10/06/2026</v>
-      </c>
-      <c r="G7" t="str">
-        <v>- Se realizará desarrollo segun orden de priorización</v>
       </c>
       <c r="H7" t="str">
         <v>- Se realizará desarrollo segun orden de priorización</v>
@@ -974,14 +974,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H3"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" customWidth="1"/>
-    <col min="5" max="5" width="16.6640625" customWidth="1"/>
-    <col min="6" max="6" width="16.6640625" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" customWidth="1"/>
-    <col min="8" max="8" width="16.6640625" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="20.33203125" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" customWidth="1"/>
+    <col min="7" max="7" width="20.33203125" customWidth="1"/>
+    <col min="8" max="8" width="20.33203125" customWidth="1"/>
     <col min="9" max="9" width="16.6640625" customWidth="1"/>
     <col min="10" max="10" width="16.6640625" customWidth="1"/>
     <col min="11" max="11" width="16.6640625" customWidth="1"/>
@@ -1051,7 +1051,7 @@
         <v>24/3/2026</v>
       </c>
       <c r="H2" t="str">
-        <v>- Se seguirá compartiendo alerta_x000d_</v>
+        <v>- Se seguirá compartiendo alerta</v>
       </c>
     </row>
     <row r="3">
@@ -1091,14 +1091,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H16"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" customWidth="1"/>
-    <col min="5" max="5" width="16.6640625" customWidth="1"/>
-    <col min="6" max="6" width="16.6640625" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" customWidth="1"/>
-    <col min="8" max="8" width="16.6640625" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="20.33203125" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" customWidth="1"/>
+    <col min="7" max="7" width="20.33203125" customWidth="1"/>
+    <col min="8" max="8" width="20.33203125" customWidth="1"/>
     <col min="9" max="9" width="16.6640625" customWidth="1"/>
     <col min="10" max="10" width="16.6640625" customWidth="1"/>
     <col min="11" max="11" width="16.6640625" customWidth="1"/>
@@ -1168,7 +1168,7 @@
         <v>03/04/2026</v>
       </c>
       <c r="H2" t="str">
-        <v>Aguardando validacion de S3._x000d_</v>
+        <v>Aguardando validacion de S3.</v>
       </c>
     </row>
     <row r="3">
@@ -1194,7 +1194,7 @@
         <v>29/04/2026</v>
       </c>
       <c r="H3" t="str">
-        <v>-S3 compartirá template en csv. -NFQ ya ha vuelto a solicitar a S3 que envíe los arquivos_x000d_</v>
+        <v>-S3 compartirá template en csv. -NFQ ya ha vuelto a solicitar a S3 que envíe los arquivos</v>
       </c>
     </row>
     <row r="4">
@@ -1220,7 +1220,7 @@
         <v>22/04/2026</v>
       </c>
       <c r="H4" t="str">
-        <v>Espernado respuesta de Operaciones de Titulos ed Renda Variavel (cliente y fecha) S3 entregará informes de Extrato Simplifcado_x000d_</v>
+        <v>Espernado respuesta de Operaciones de Titulos ed Renda Variavel (cliente y fecha) S3 entregará informes de Extrato Simplifcado</v>
       </c>
     </row>
     <row r="5">
@@ -1246,7 +1246,7 @@
         <v>29/04/2026</v>
       </c>
       <c r="H5" t="str">
-        <v>- Validación de lado S3 para promocionar a UAT_x000d_</v>
+        <v>- Validación de lado S3 para promocionar a UAT</v>
       </c>
     </row>
     <row r="6">
@@ -1272,7 +1272,7 @@
         <v>07/07/2025</v>
       </c>
       <c r="H6" t="str">
-        <v>Validación de lado S3_x000d_</v>
+        <v>Validación de lado S3</v>
       </c>
     </row>
     <row r="7">
@@ -1298,7 +1298,7 @@
         <v>05/09/2025</v>
       </c>
       <c r="H7" t="str">
-        <v>Validación de lado S3_x000d_</v>
+        <v>Validación de lado S3</v>
       </c>
     </row>
     <row r="8">
@@ -1324,7 +1324,7 @@
         <v>28/10/2025</v>
       </c>
       <c r="H8" t="str">
-        <v>Validación de lado S3_x000d_</v>
+        <v>Validación de lado S3</v>
       </c>
     </row>
     <row r="9">
@@ -1350,7 +1350,7 @@
         <v>28/10/2025</v>
       </c>
       <c r="H9" t="str">
-        <v>Validación de lado S3_x000d_</v>
+        <v>Validación de lado S3</v>
       </c>
     </row>
     <row r="10">
@@ -1376,7 +1376,7 @@
         <v>31/10/2025</v>
       </c>
       <c r="H10" t="str">
-        <v>Validación de lado S3_x000d_</v>
+        <v>Validación de lado S3</v>
       </c>
     </row>
     <row r="11">
@@ -1402,7 +1402,7 @@
         <v>21/01/2026</v>
       </c>
       <c r="H11" t="str">
-        <v>Validación de lado S3_x000d_</v>
+        <v>Validación de lado S3</v>
       </c>
     </row>
     <row r="12">
@@ -1428,7 +1428,7 @@
         <v>28/01/2026</v>
       </c>
       <c r="H12" t="str">
-        <v>Validación de lado S3_x000d_</v>
+        <v>Validación de lado S3</v>
       </c>
     </row>
     <row r="13">
@@ -1454,7 +1454,7 @@
         <v>31/10/2025</v>
       </c>
       <c r="H13" t="str">
-        <v>- S3 junto con NFQ revisará ambiente, a la espera de activación al equipo de projeto_x000d_</v>
+        <v>- S3 junto con NFQ revisará ambiente, a la espera de activación al equipo de projeto.</v>
       </c>
     </row>
     <row r="14">
@@ -1480,7 +1480,7 @@
         <v>21/01/2026</v>
       </c>
       <c r="H14" t="str">
-        <v>- S3 notificará resultados de validaciones_x000d_</v>
+        <v>- S3 notificará resultados de validaciones_</v>
       </c>
     </row>
     <row r="15">
@@ -1506,7 +1506,7 @@
         <v>29/01/2026</v>
       </c>
       <c r="H15" t="str">
-        <v>- S3 validará arreglos en los informes. - S3 compartirá detalles de PS para poder dar suporte._x000d_</v>
+        <v>- S3 validará arreglos en los informes. - S3 compartirá detalles de PS para poder dar suporte.</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
PPT - 17/06/2026 - Final
</commit_message>
<xml_diff>
--- a/dashboard_data_template.xlsx
+++ b/dashboard_data_template.xlsx
@@ -539,10 +539,10 @@
         <v>Ajuste Proceso de Carga</v>
       </c>
       <c r="B5" t="str">
-        <v>En proceso</v>
+        <v>Completado</v>
       </c>
       <c r="C5" t="str">
-        <v>UAT</v>
+        <v>PRD</v>
       </c>
       <c r="D5" t="str">
         <v>NFQ / S3</v>

</xml_diff>